<commit_message>
docs: align NPV and Plan Excel files with the HSU course registration system project context
</commit_message>
<xml_diff>
--- a/Ebooks/NPV - Students.xlsx
+++ b/Ebooks/NPV - Students.xlsx
@@ -1,36 +1,100 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hoa Sen\Project Management\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D074DDC3-FD4B-4563-A327-7F937E126029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1E71F62E-CCC1-41A3-BE73-8F04C42DD365}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Example" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Example</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>admin</dc:creator>
+  <cp:lastModifiedBy>SON Nguyen Van</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2023-08-02T14:34:12Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2024-07-26T02:47:01Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
+<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <c r="G11" i="1" l="1"/>
+  <c r="B11" i="1"/>
+  <c r="B12" i="1"/>
+  <c r="C21" i="1"/>
+  <c r="D21" i="1"/>
+  <c r="E21" i="1"/>
+  <c r="F21" i="1"/>
+  <c r="B21" i="1"/>
+  <c r="C20" i="1"/>
+  <c r="D20" i="1"/>
+  <c r="E20" i="1"/>
+  <c r="F20" i="1"/>
+  <c r="B20" i="1"/>
+  <c r="B9" i="1"/>
+  <c r="G9" i="1" s="1"/>
+  <c r="B8" i="1"/>
+  <c r="G8" i="1" s="1"/>
+  <c r="C9" i="1"/>
+  <c r="D9" i="1"/>
+  <c r="E9" i="1"/>
+  <c r="F9" i="1"/>
+  <c r="C8" i="1"/>
+  <c r="D8" i="1"/>
+  <c r="E8" i="1"/>
+  <c r="F8" i="1"/>
+  <c r="G17" i="1"/>
+  <c r="G16" i="1"/>
+  <c r="G5" i="1"/>
+  <c r="G4" i="1"/>
+  <c r="C18" i="1"/>
+  <c r="D18" i="1"/>
+  <c r="E18" i="1"/>
+  <c r="F18" i="1"/>
+  <c r="B18" i="1"/>
+  <c r="C6" i="1"/>
+  <c r="D6" i="1"/>
+  <c r="E6" i="1"/>
+  <c r="F6" i="1"/>
+  <c r="B6" i="1"/>
+  <c r="G21" i="1" l="1"/>
+  <c r="G20" i="1"/>
+  <c r="B25" i="1" s="1"/>
+  <c r="C11" i="1"/>
+  <c r="B23" i="1"/>
+  <c r="G6" i="1"/>
+  <c r="G18" i="1"/>
+  <c r="C23" i="1" l="1"/>
+</calcChain>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
-    <t>Distcount rate</t>
-  </si>
-  <si>
-    <t>Project 1</t>
+    <t>Discount rate</t>
+  </si>
+  <si>
+    <t>HSU Course Portal Project</t>
   </si>
   <si>
     <t>Benefits</t>
@@ -57,7 +121,7 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Project 2</t>
+    <t>Legacy Upgrade Alternative</t>
   </si>
   <si>
     <t>Cash flow</t>
@@ -86,7 +150,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
@@ -196,7 +260,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -491,7 +555,32 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hoa Sen\Project Management\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D074DDC3-FD4B-4563-A327-7F937E126029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1E71F62E-CCC1-41A3-BE73-8F04C42DD365}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Example" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75F1F0F4-63CA-4B2F-8BD0-FC5A0276C0D1}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -504,7 +593,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -555,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="C4" s="2">
-        <v>2000</v>
+        <v>200000</v>
       </c>
       <c r="D4" s="2">
-        <v>3000</v>
+        <v>200000</v>
       </c>
       <c r="E4" s="2">
-        <v>4000</v>
+        <v>200000</v>
       </c>
       <c r="F4" s="2">
-        <v>5000</v>
+        <v>200000</v>
       </c>
       <c r="G4" s="2">
         <f>SUM(B4:F4)</f>
@@ -576,19 +665,19 @@
         <v>15</v>
       </c>
       <c r="B5" s="2">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="C5" s="2">
-        <v>1000</v>
+        <v>40000</v>
       </c>
       <c r="D5" s="2">
-        <v>1000</v>
+        <v>40000</v>
       </c>
       <c r="E5" s="2">
-        <v>1000</v>
+        <v>40000</v>
       </c>
       <c r="F5" s="2">
-        <v>1000</v>
+        <v>40000</v>
       </c>
       <c r="G5" s="2">
         <f>SUM(B5:F5)</f>
@@ -787,19 +876,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="2">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="C16" s="2">
-        <v>2000</v>
+        <v>80000</v>
       </c>
       <c r="D16" s="2">
-        <v>4000</v>
+        <v>80000</v>
       </c>
       <c r="E16" s="2">
-        <v>4000</v>
+        <v>80000</v>
       </c>
       <c r="F16" s="2">
-        <v>4000</v>
+        <v>80000</v>
       </c>
       <c r="G16" s="2">
         <f>SUM(B16:F16)</f>
@@ -811,19 +900,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="2">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="C17" s="2">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D17" s="2">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E17" s="2">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="F17" s="2">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" ref="G17:G18" si="3">SUM(B17:F17)</f>

</xml_diff>